<commit_message>
Added scrollable state to threats
</commit_message>
<xml_diff>
--- a/backend/Blockchain/leader/alerts.xlsx
+++ b/backend/Blockchain/leader/alerts.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,46 +413,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Threat ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Source IP</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Attack</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Target IP</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Start Time</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Attack Count</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
@@ -2099,6 +2087,462 @@
         <v>1</v>
       </c>
       <c r="H44" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:47:43</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>9</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:47:54</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>7</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:48:19</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>8</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>XSS</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:50:22</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:58:28</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>54</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:58:31</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>66</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:58:25</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>33</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:58:28</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>64</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-05-02T22:58:31</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>53</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Keylogging</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-05-02T23:00:30</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-05-02T23:00:56</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Credential Harvesting</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>data exfiltration</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-05-02T23:01:56</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" t="inlineStr">
         <is>
           <t>low</t>
         </is>

</xml_diff>

<commit_message>
Changes made to 2 cards and a graph in Overview.js
</commit_message>
<xml_diff>
--- a/backend/Blockchain/leader/alerts.xlsx
+++ b/backend/Blockchain/leader/alerts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2548,6 +2548,196 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-05-03T13:50:12</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>19</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-05-03T13:50:12</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>23</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-05-03T13:53:29</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-05-03T13:54:18</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Cookie Stealing</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>data exfiltration</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-05-03T13:55:00</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
registered alert logs in Overview and Threats
</commit_message>
<xml_diff>
--- a/backend/Blockchain/leader/alerts.xlsx
+++ b/backend/Blockchain/leader/alerts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2738,6 +2738,766 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-05-03T21:56:38</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>150</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-05-03T21:56:37</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>131</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-05-03T21:56:56</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>150</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-05-03T21:56:55</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>150</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>XSS</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-05-03T21:58:35</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-05-03T21:59:25</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Keylogging</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:01:36</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>2</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:03:03</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>18</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:04:29</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>100</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:04:29</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>100</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Cookie Stealing</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>data exfiltration</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:06:23</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>2</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:16</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>7</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>authentication</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:07:16</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>25</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:38</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>160</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:41</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>40</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DoS</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:08:38</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>176</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:46</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:18:51</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:20:05</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>2</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Session Hijacking</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>social enginnering</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>192.168.29.124</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-05-03T22:21:24</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>